<commit_message>
Sdn 134 135/improvement/separate projects (#151)
* refactor(scope): extract Trucks as standalone app, remove all Tickets code

Separated the monorepo into a Trucks-only application by removing all
Acarreos/Gasolina/Concreto/Asfalto ticket subsystems — routes, components,
stores, printer schemas, CSV schemas, and API endpoints. Relocated all truck
routes from /trucks/* to the app root (/, /db, /dashboard, /materials, /users,
/voucher), updated middleware access-control and post-login redirects per role,
and wired up full Frente management (add/edit/delete/logo) into TrucksDbHeader
and a new FrentesManagerSheet accessible from the sidebar for owners.
Brand color palette (green/gold/wine) applied consistently across all Frente
dialogs.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

* add new test metadatacamion file

---------

Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/test_metadatacamion.xlsx
+++ b/public/documents/test_metadatacamion.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C793DB7-5FF3-47CE-8649-C5DC98B303EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4FA2748-982D-4E81-919A-3D18F5CE7F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{32B9423A-B4F8-4DEF-99A3-E731A16C4C3A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{32B9423A-B4F8-4DEF-99A3-E731A16C4C3A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029" iterate="1" iterateCount="20000"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -96,93 +96,6 @@
     <t>Operador2</t>
   </si>
   <si>
-    <t>T1F1</t>
-  </si>
-  <si>
-    <t>T2F2</t>
-  </si>
-  <si>
-    <t>T1F2</t>
-  </si>
-  <si>
-    <t>T2F3</t>
-  </si>
-  <si>
-    <t>T1F3</t>
-  </si>
-  <si>
-    <t>T2F4</t>
-  </si>
-  <si>
-    <t>T1F4</t>
-  </si>
-  <si>
-    <t>T2F5</t>
-  </si>
-  <si>
-    <t>T1F5</t>
-  </si>
-  <si>
-    <t>T2F6</t>
-  </si>
-  <si>
-    <t>T1F6</t>
-  </si>
-  <si>
-    <t>T2F7</t>
-  </si>
-  <si>
-    <t>T1F7</t>
-  </si>
-  <si>
-    <t>T2F8</t>
-  </si>
-  <si>
-    <t>T1F8</t>
-  </si>
-  <si>
-    <t>T2F9</t>
-  </si>
-  <si>
-    <t>T1F9</t>
-  </si>
-  <si>
-    <t>T2F10</t>
-  </si>
-  <si>
-    <t>T1F10</t>
-  </si>
-  <si>
-    <t>T2F11</t>
-  </si>
-  <si>
-    <t>T1F11</t>
-  </si>
-  <si>
-    <t>T2F12</t>
-  </si>
-  <si>
-    <t>T1F12</t>
-  </si>
-  <si>
-    <t>T2F13</t>
-  </si>
-  <si>
-    <t>T1F13</t>
-  </si>
-  <si>
-    <t>T2F14</t>
-  </si>
-  <si>
-    <t>T1F14</t>
-  </si>
-  <si>
-    <t>T2F15</t>
-  </si>
-  <si>
-    <t>T1F15</t>
-  </si>
-  <si>
     <t>Operador3</t>
   </si>
   <si>
@@ -394,6 +307,93 @@
   </si>
   <si>
     <t>Localidad14</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F1</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F2</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F3</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F4</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F5</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F6</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F7</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F8</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F9</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F10</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F11</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F12</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F13</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F14</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F15</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F16</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F17</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F18</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F19</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F20</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F21</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F22</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F23</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F24</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F25</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F26</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F27</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F28</t>
+  </si>
+  <si>
+    <t>TPCDMXP-F29</t>
   </si>
 </sst>
 </file>
@@ -441,11 +441,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -761,15 +764,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{335DF882-D054-4F59-944C-F3D0F4E5F17D}">
   <dimension ref="A1:J30"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="42.6328125" customWidth="1"/>
-    <col min="5" max="5" width="16.1796875" customWidth="1"/>
+    <col min="2" max="2" width="42.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="16.21875" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="10" max="10" width="26.453125" customWidth="1"/>
+    <col min="10" max="10" width="26.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -795,10 +799,10 @@
         <v>14</v>
       </c>
       <c r="J1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -808,8 +812,8 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
-        <v>19</v>
+      <c r="D2" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>9</v>
@@ -818,16 +822,16 @@
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="H2">
         <v>123456</v>
       </c>
       <c r="J2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -837,8 +841,8 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>20</v>
+      <c r="D3" s="4" t="s">
+        <v>91</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>9</v>
@@ -847,27 +851,27 @@
         <v>15</v>
       </c>
       <c r="G3" t="s">
-        <v>76</v>
+        <v>47</v>
       </c>
       <c r="H3" s="3">
         <v>123456</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>21</v>
+      <c r="D4" s="4" t="s">
+        <v>92</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>9</v>
@@ -876,27 +880,27 @@
         <v>15</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="H4" s="3">
         <v>123456</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>22</v>
+      <c r="D5" s="4" t="s">
+        <v>93</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>9</v>
@@ -905,27 +909,27 @@
         <v>15</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="H5" s="3">
         <v>123456</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>23</v>
+      <c r="D6" s="4" t="s">
+        <v>94</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>9</v>
@@ -934,27 +938,27 @@
         <v>15</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="H6" s="3">
         <v>123456</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>24</v>
+      <c r="D7" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>9</v>
@@ -963,27 +967,27 @@
         <v>15</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="H7" s="3">
         <v>123456</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>25</v>
+      <c r="D8" s="4" t="s">
+        <v>96</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>9</v>
@@ -992,27 +996,27 @@
         <v>15</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>81</v>
+        <v>52</v>
       </c>
       <c r="H8" s="3">
         <v>123456</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>26</v>
+      <c r="D9" s="4" t="s">
+        <v>97</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>9</v>
@@ -1021,27 +1025,27 @@
         <v>17</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="H9" s="3">
         <v>123456</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>27</v>
+      <c r="D10" s="4" t="s">
+        <v>98</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>9</v>
@@ -1050,27 +1054,27 @@
         <v>17</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>83</v>
+        <v>54</v>
       </c>
       <c r="H10" s="3">
         <v>123456</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>28</v>
+      <c r="D11" s="4" t="s">
+        <v>99</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>9</v>
@@ -1079,27 +1083,27 @@
         <v>17</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="H11" s="3">
         <v>123456</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>29</v>
+      <c r="D12" s="4" t="s">
+        <v>100</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>9</v>
@@ -1108,27 +1112,27 @@
         <v>17</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>85</v>
+        <v>56</v>
       </c>
       <c r="H12" s="3">
         <v>123456</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>30</v>
+      <c r="D13" s="4" t="s">
+        <v>101</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>10</v>
@@ -1137,27 +1141,27 @@
         <v>17</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="H13" s="3">
         <v>123456</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>31</v>
+      <c r="D14" s="4" t="s">
+        <v>102</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>10</v>
@@ -1166,27 +1170,27 @@
         <v>17</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="H14" s="3">
         <v>123456</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>32</v>
+      <c r="D15" s="4" t="s">
+        <v>103</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>10</v>
@@ -1195,27 +1199,27 @@
         <v>17</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="H15" s="3">
         <v>123456</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="C16">
         <v>2</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>33</v>
+      <c r="D16" s="4" t="s">
+        <v>104</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>10</v>
@@ -1224,7 +1228,7 @@
         <v>17</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="H16" s="3">
         <v>123456</v>
@@ -1233,18 +1237,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>34</v>
+      <c r="D17" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>10</v>
@@ -1253,7 +1257,7 @@
         <v>17</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="H17" s="3">
         <v>123456</v>
@@ -1262,18 +1266,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>35</v>
+      <c r="D18" s="4" t="s">
+        <v>106</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>10</v>
@@ -1282,7 +1286,7 @@
         <v>16</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>91</v>
+        <v>62</v>
       </c>
       <c r="H18" s="3">
         <v>123456</v>
@@ -1291,18 +1295,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>36</v>
+      <c r="D19" s="4" t="s">
+        <v>107</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>10</v>
@@ -1311,7 +1315,7 @@
         <v>16</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>92</v>
+        <v>63</v>
       </c>
       <c r="H19" s="3">
         <v>123456</v>
@@ -1320,18 +1324,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="C20">
         <v>2</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>37</v>
+      <c r="D20" s="4" t="s">
+        <v>108</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>10</v>
@@ -1340,7 +1344,7 @@
         <v>16</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="H20" s="3">
         <v>123456</v>
@@ -1349,18 +1353,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="C21">
         <v>2</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>38</v>
+      <c r="D21" s="4" t="s">
+        <v>109</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>10</v>
@@ -1369,7 +1373,7 @@
         <v>16</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>94</v>
+        <v>65</v>
       </c>
       <c r="H21" s="3">
         <v>123456</v>
@@ -1378,18 +1382,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="C22">
         <v>2</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>39</v>
+      <c r="D22" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>10</v>
@@ -1398,7 +1402,7 @@
         <v>16</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="H22" s="3">
         <v>123456</v>
@@ -1407,18 +1411,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>40</v>
+      <c r="D23" s="4" t="s">
+        <v>111</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>10</v>
@@ -1427,7 +1431,7 @@
         <v>16</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>96</v>
+        <v>67</v>
       </c>
       <c r="H23" s="3">
         <v>123456</v>
@@ -1436,18 +1440,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="C24">
         <v>2</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>41</v>
+      <c r="D24" s="4" t="s">
+        <v>112</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>11</v>
@@ -1456,7 +1460,7 @@
         <v>16</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="H24" s="3">
         <v>123456</v>
@@ -1465,18 +1469,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>42</v>
+      <c r="D25" s="4" t="s">
+        <v>113</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>11</v>
@@ -1485,7 +1489,7 @@
         <v>16</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="H25" s="3">
         <v>123456</v>
@@ -1494,18 +1498,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C26">
         <v>2</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>43</v>
+      <c r="D26" s="4" t="s">
+        <v>114</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>11</v>
@@ -1514,7 +1518,7 @@
         <v>17</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="H26" s="3">
         <v>123456</v>
@@ -1523,18 +1527,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="C27">
         <v>2</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>44</v>
+      <c r="D27" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>11</v>
@@ -1543,7 +1547,7 @@
         <v>17</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="H27" s="3">
         <v>123456</v>
@@ -1552,18 +1556,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>45</v>
+      <c r="D28" s="4" t="s">
+        <v>116</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>11</v>
@@ -1572,7 +1576,7 @@
         <v>17</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="H28" s="3">
         <v>123456</v>
@@ -1581,18 +1585,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="C29">
         <v>2</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>46</v>
+      <c r="D29" s="4" t="s">
+        <v>117</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>11</v>
@@ -1601,7 +1605,7 @@
         <v>17</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="H29" s="3">
         <v>123456</v>
@@ -1610,18 +1614,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>74</v>
+        <v>45</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
-      <c r="D30" s="3" t="s">
-        <v>47</v>
+      <c r="D30" s="4" t="s">
+        <v>118</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>11</v>
@@ -1630,7 +1634,7 @@
         <v>17</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="H30" s="3">
         <v>123456</v>

</xml_diff>